<commit_message>
jacobs retail prices - first update
</commit_message>
<xml_diff>
--- a/Data/electricity_tariffs_july_25.xlsx
+++ b/Data/electricity_tariffs_july_25.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unimelbcloud-my.sharepoint.com/personal/dominic_jones_grattaninstitute_edu_au/Documents/Energy/Analysis/analysis_cp_dj_2025/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7CEED8F1-813D-4156-91F0-2CE7A2B20F14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="8_{7CEED8F1-813D-4156-91F0-2CE7A2B20F14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A64D9B44-9513-44BE-8AC4-DFC3E7D792E8}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A003514B-5DDD-4994-A84B-CB9D3FD32C4E}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="28">
   <si>
     <t>State</t>
   </si>
@@ -114,6 +114,12 @@
   </si>
   <si>
     <t>Synergy</t>
+  </si>
+  <si>
+    <t>ACT</t>
+  </si>
+  <si>
+    <t>Origin go variable</t>
   </si>
 </sst>
 </file>
@@ -519,7 +525,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19DE869E-D0B0-4ECD-A9BF-8A8297012797}">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.375" customWidth="1"/>
@@ -790,6 +796,34 @@
         <v>46.141199999999998</v>
       </c>
     </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D14" t="s">
+        <v>27</v>
+      </c>
+      <c r="E14" t="s">
+        <v>6</v>
+      </c>
+      <c r="F14">
+        <v>111.55</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E15" t="s">
+        <v>7</v>
+      </c>
+      <c r="F15">
+        <v>26.64</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="D4" r:id="rId1" display="https://www.energymadeeasy.gov.au/plan?id=ORI887900MRE4&amp;postcode=4000&amp;pricingPeriod=yearly&amp;withDiscounts=false&amp;benchmarkUsage=medium" xr:uid="{4B9504E6-0C2F-4467-8232-1C5B4B1A79A1}"/>

</xml_diff>